<commit_message>
Added a rough draft for the database.
</commit_message>
<xml_diff>
--- a/Database/EldenBosses.xlsx
+++ b/Database/EldenBosses.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\OneDrive\Documents\TheEldenLords\Extra Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\College\ETSU\Spring 2026\Server Side Programming\TheEldenLords\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8ADE5E9-5454-4507-A7CC-990C9272980A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE012AE-CB08-4C57-9AB2-210352564E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="10425" windowHeight="13403" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,28 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="91">
-  <si>
-    <t>Bosses</t>
-  </si>
-  <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>Lore</t>
-  </si>
-  <si>
-    <t>Stats</t>
-  </si>
-  <si>
-    <t>Prerequisites</t>
-  </si>
-  <si>
-    <t>Help</t>
-  </si>
-  <si>
-    <t>Rewards</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="84">
   <si>
     <t>Margit The Fell Omen</t>
   </si>
@@ -615,359 +594,336 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.796875" customWidth="1"/>
-    <col min="2" max="2" width="22.1328125" customWidth="1"/>
-    <col min="3" max="3" width="26.53125" customWidth="1"/>
-    <col min="4" max="4" width="67.3984375" customWidth="1"/>
-    <col min="5" max="5" width="56.9296875" customWidth="1"/>
-    <col min="6" max="6" width="70.53125" customWidth="1"/>
-    <col min="7" max="7" width="70.06640625" customWidth="1"/>
+    <col min="1" max="1" width="34.77734375" customWidth="1"/>
+    <col min="2" max="2" width="22.109375" customWidth="1"/>
+    <col min="3" max="3" width="26.5546875" customWidth="1"/>
+    <col min="4" max="4" width="67.44140625" customWidth="1"/>
+    <col min="5" max="5" width="56.88671875" customWidth="1"/>
+    <col min="6" max="6" width="70.5546875" customWidth="1"/>
+    <col min="7" max="7" width="70.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>8</v>
       </c>
       <c r="B3" t="s">
         <v>22</v>
       </c>
       <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" t="s">
         <v>27</v>
       </c>
-      <c r="E3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s">
         <v>35</v>
       </c>
-      <c r="G3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+      <c r="E5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4" t="s">
-        <v>34</v>
-      </c>
-      <c r="G4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+      <c r="B10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" t="s">
-        <v>39</v>
-      </c>
-      <c r="F5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E6" t="s">
-        <v>45</v>
-      </c>
-      <c r="F6" t="s">
-        <v>43</v>
-      </c>
-      <c r="G6" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D7" t="s">
-        <v>47</v>
-      </c>
-      <c r="E7" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" t="s">
-        <v>53</v>
-      </c>
-      <c r="E8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" t="s">
-        <v>51</v>
-      </c>
-      <c r="G8" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F9" t="s">
-        <v>56</v>
-      </c>
-      <c r="G9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E10" t="s">
-        <v>61</v>
-      </c>
-      <c r="F10" t="s">
-        <v>59</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="B11" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" t="s">
-        <v>62</v>
       </c>
       <c r="D11" t="s">
         <v>63</v>
       </c>
       <c r="E11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>64</v>
       </c>
-      <c r="F11" t="s">
+      <c r="B12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" t="s">
         <v>65</v>
       </c>
-      <c r="G11" t="s">
+      <c r="E12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="G12" t="s">
         <v>67</v>
       </c>
-      <c r="D12" t="s">
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G13" t="s">
         <v>70</v>
       </c>
-      <c r="E12" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" t="s">
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
         <v>68</v>
       </c>
-      <c r="G12" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>71</v>
-      </c>
-      <c r="B13" t="s">
-        <v>67</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="D14" t="s">
         <v>72</v>
       </c>
-      <c r="E13" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="E14" t="s">
         <v>73</v>
       </c>
-      <c r="G13" t="s">
+      <c r="F14" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="G14" t="s">
         <v>75</v>
       </c>
-      <c r="D14" t="s">
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" t="s">
+        <v>76</v>
+      </c>
+      <c r="E15" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" t="s">
         <v>78</v>
       </c>
-      <c r="E14" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" t="s">
-        <v>76</v>
-      </c>
-      <c r="G14" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" t="s">
-        <v>75</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="G15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16" t="s">
+        <v>82</v>
+      </c>
+      <c r="E16" t="s">
+        <v>81</v>
+      </c>
+      <c r="F16" t="s">
+        <v>80</v>
+      </c>
+      <c r="G16" t="s">
         <v>79</v>
-      </c>
-      <c r="E15" t="s">
-        <v>80</v>
-      </c>
-      <c r="F15" t="s">
-        <v>81</v>
-      </c>
-      <c r="G15" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" t="s">
-        <v>90</v>
-      </c>
-      <c r="D16" t="s">
-        <v>83</v>
-      </c>
-      <c r="E16" t="s">
-        <v>84</v>
-      </c>
-      <c r="F16" t="s">
-        <v>85</v>
-      </c>
-      <c r="G16" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" t="s">
-        <v>90</v>
-      </c>
-      <c r="D17" t="s">
-        <v>89</v>
-      </c>
-      <c r="E17" t="s">
-        <v>88</v>
-      </c>
-      <c r="F17" t="s">
-        <v>87</v>
-      </c>
-      <c r="G17" t="s">
-        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>